<commit_message>
added demo data and modular changes
</commit_message>
<xml_diff>
--- a/public/bulk-order-template.xlsx
+++ b/public/bulk-order-template.xlsx
@@ -399,31 +399,6 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:W4"/>
-  <cols>
-    <col min="1" max="1" width="14.83203125" customWidth="1"/>
-    <col min="2" max="2" width="15.83203125" customWidth="1"/>
-    <col min="3" max="3" width="14.83203125" customWidth="1"/>
-    <col min="4" max="4" width="12.83203125" customWidth="1"/>
-    <col min="5" max="5" width="17.83203125" customWidth="1"/>
-    <col min="6" max="6" width="12.83203125" customWidth="1"/>
-    <col min="7" max="7" width="16.83203125" customWidth="1"/>
-    <col min="8" max="8" width="16.83203125" customWidth="1"/>
-    <col min="9" max="9" width="12.83203125" customWidth="1"/>
-    <col min="10" max="10" width="12.83203125" customWidth="1"/>
-    <col min="11" max="11" width="12.83203125" customWidth="1"/>
-    <col min="12" max="12" width="12.83203125" customWidth="1"/>
-    <col min="13" max="13" width="12.83203125" customWidth="1"/>
-    <col min="14" max="14" width="14.83203125" customWidth="1"/>
-    <col min="15" max="15" width="12.83203125" customWidth="1"/>
-    <col min="16" max="16" width="12.83203125" customWidth="1"/>
-    <col min="17" max="17" width="12.83203125" customWidth="1"/>
-    <col min="18" max="18" width="12.83203125" customWidth="1"/>
-    <col min="19" max="19" width="13.83203125" customWidth="1"/>
-    <col min="20" max="20" width="14.83203125" customWidth="1"/>
-    <col min="21" max="21" width="13.83203125" customWidth="1"/>
-    <col min="22" max="22" width="14.83203125" customWidth="1"/>
-    <col min="23" max="23" width="12.83203125" customWidth="1"/>
-  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -718,11 +693,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B10"/>
-  <cols>
-    <col min="1" max="1" width="20.83203125" customWidth="1"/>
-    <col min="2" max="2" width="110.83203125" customWidth="1"/>
-  </cols>
+  <dimension ref="A1:B11"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -742,7 +713,7 @@
         <v>Multiple products</v>
       </c>
       <c r="B4" t="str">
-        <v>Repeat the same Order number on several rows. Customer, payment and package columns are read from the first row of that order.</v>
+        <v>Repeat the same Order number on several rows (one row per product, maximum 5 products per order). Customer, payment and package columns are read from the first row of that order.</v>
       </c>
     </row>
     <row r="5">
@@ -787,15 +758,23 @@
     </row>
     <row r="10">
       <c r="A10" t="str">
+        <v>Product limit</v>
+      </c>
+      <c r="B10" t="str">
+        <v>An order can contain at most 5 products. A sheet with more than 5 rows for one order number is rejected for that order.</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="str">
         <v>Note</v>
       </c>
-      <c r="B10" t="str">
+      <c r="B11" t="str">
         <v>Delete the sample rows before uploading your own orders. Keep the header row unchanged.</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:B10"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:B11"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>